<commit_message>
setup 1-3 updates, setup 4-6 results
</commit_message>
<xml_diff>
--- a/data/aadt.xlsx
+++ b/data/aadt.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\GitHub\braess-paradox-sp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B8D98FE4-75A5-416D-A153-1664C17BC5E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51E23FD3-B19C-4FD4-97FE-F8ECA0ADD613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{A875B457-C1A5-40D5-BC91-583C5F2977DC}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{A875B457-C1A5-40D5-BC91-583C5F2977DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="71">
   <si>
     <t>Name</t>
   </si>
@@ -135,6 +135,120 @@
   </si>
   <si>
     <t>La Paz Deep Sea Water Port Rd</t>
+  </si>
+  <si>
+    <t>Road Section ID</t>
+  </si>
+  <si>
+    <t>S00081PN</t>
+  </si>
+  <si>
+    <t>S00085PN</t>
+  </si>
+  <si>
+    <t>S00075PN</t>
+  </si>
+  <si>
+    <t>S00079PN</t>
+  </si>
+  <si>
+    <t>S00488PN</t>
+  </si>
+  <si>
+    <t>S00086PN</t>
+  </si>
+  <si>
+    <t>S00021PN</t>
+  </si>
+  <si>
+    <t>S00044PN</t>
+  </si>
+  <si>
+    <t>S00425PN</t>
+  </si>
+  <si>
+    <t>S00093PN</t>
+  </si>
+  <si>
+    <t>S00503PN</t>
+  </si>
+  <si>
+    <t>S00065PN</t>
+  </si>
+  <si>
+    <t>S00003PN</t>
+  </si>
+  <si>
+    <t>S00495PN</t>
+  </si>
+  <si>
+    <t>S0508PN</t>
+  </si>
+  <si>
+    <t>S00084PN</t>
+  </si>
+  <si>
+    <t>S00078PN</t>
+  </si>
+  <si>
+    <t>S00493PN</t>
+  </si>
+  <si>
+    <t>S00507PN</t>
+  </si>
+  <si>
+    <t>S00019PN</t>
+  </si>
+  <si>
+    <t>S00071PN</t>
+  </si>
+  <si>
+    <t>S00053PN</t>
+  </si>
+  <si>
+    <t>S00064PN</t>
+  </si>
+  <si>
+    <t>S00494PN</t>
+  </si>
+  <si>
+    <t>S00505PN</t>
+  </si>
+  <si>
+    <t>S00500PN</t>
+  </si>
+  <si>
+    <t>S00491PN</t>
+  </si>
+  <si>
+    <t>S00016PN</t>
+  </si>
+  <si>
+    <t>S00506PN</t>
+  </si>
+  <si>
+    <t>S00060PN</t>
+  </si>
+  <si>
+    <t>S00080PN</t>
+  </si>
+  <si>
+    <t>S00486PN</t>
+  </si>
+  <si>
+    <t>S00483PN</t>
+  </si>
+  <si>
+    <t>S00063PN</t>
+  </si>
+  <si>
+    <t>S00049PN</t>
+  </si>
+  <si>
+    <t>S00062PN</t>
+  </si>
+  <si>
+    <t>S00077PN</t>
   </si>
 </sst>
 </file>
@@ -506,354 +620,489 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1623E3E9-9CAF-4511-B3BA-95B0DB4104C8}">
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="36" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2">
+        <v>37299</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3">
+        <v>34899</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4">
+        <v>32322</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5">
+        <v>28471</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6">
+        <v>28363</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7">
+        <v>27677</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8">
+        <v>27480</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9">
+        <v>26847</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10">
+        <v>25643</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11">
+        <v>24186</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12">
+        <v>22497</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13">
+        <v>21760</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>2</v>
       </c>
-      <c r="B2">
+      <c r="B14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14">
         <v>20650</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3">
-        <v>22497</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>14268</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5">
-        <v>10734</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6">
-        <v>3810</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7">
-        <v>13282</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8">
-        <v>19590</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9">
-        <v>24186</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10">
-        <v>11833</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11">
-        <v>17354</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12">
-        <v>15088</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13">
-        <v>27677</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14">
-        <v>21760</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>12</v>
       </c>
-      <c r="B15">
+      <c r="B15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15">
         <v>19944</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16">
+        <v>19590</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17">
+        <v>18208</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18">
+        <v>18208</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>3</v>
       </c>
-      <c r="B16">
+      <c r="B19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19">
         <v>17846</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>11</v>
-      </c>
-      <c r="B17">
-        <v>26847</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>13</v>
-      </c>
-      <c r="B18">
-        <v>25643</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B19">
-        <v>34899</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>9</v>
-      </c>
-      <c r="B20">
-        <v>14031</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="B20" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20">
+        <v>17354</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>8</v>
-      </c>
-      <c r="B21">
-        <v>32322</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="B21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C21">
+        <v>17166</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B22">
-        <v>37299</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+      <c r="B22" t="s">
+        <v>67</v>
+      </c>
+      <c r="C22">
+        <v>16771</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>11</v>
-      </c>
-      <c r="B23">
-        <v>28363</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="B23" t="s">
+        <v>63</v>
+      </c>
+      <c r="C23">
+        <v>15522</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>9</v>
       </c>
-      <c r="B24">
+      <c r="B24" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24">
         <v>15398</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>14</v>
-      </c>
-      <c r="B25">
-        <v>15522</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+      <c r="B25" t="s">
+        <v>53</v>
+      </c>
+      <c r="C25">
+        <v>15088</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26">
+        <v>14268</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27">
+        <v>14031</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>5</v>
+      </c>
+      <c r="B28" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28">
+        <v>13282</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>25</v>
+      </c>
+      <c r="B29" t="s">
+        <v>37</v>
+      </c>
+      <c r="C29">
+        <v>12573</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>8</v>
+      </c>
+      <c r="B30" t="s">
+        <v>52</v>
+      </c>
+      <c r="C30">
+        <v>11833</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>24</v>
+      </c>
+      <c r="B31" t="s">
+        <v>36</v>
+      </c>
+      <c r="C31">
+        <v>11821</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>3</v>
+      </c>
+      <c r="B32" t="s">
+        <v>48</v>
+      </c>
+      <c r="C32">
+        <v>10734</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>44</v>
+      </c>
+      <c r="C33">
+        <v>10090</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34">
+        <v>6317</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>19</v>
+      </c>
+      <c r="B35" t="s">
+        <v>68</v>
+      </c>
+      <c r="C35">
+        <v>6113</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B36" t="s">
+        <v>42</v>
+      </c>
+      <c r="C36">
+        <v>5704</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>22</v>
+      </c>
+      <c r="B37" t="s">
+        <v>34</v>
+      </c>
+      <c r="C37">
+        <v>5034</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>4</v>
+      </c>
+      <c r="B38" t="s">
+        <v>49</v>
+      </c>
+      <c r="C38">
+        <v>3810</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>20</v>
+      </c>
+      <c r="B39" t="s">
+        <v>69</v>
+      </c>
+      <c r="C39">
+        <v>3323</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>21</v>
+      </c>
+      <c r="B40" t="s">
+        <v>70</v>
+      </c>
+      <c r="C40">
+        <v>1801</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>26</v>
+      </c>
+      <c r="B41" t="s">
+        <v>38</v>
+      </c>
+      <c r="C41">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>23</v>
+      </c>
+      <c r="B42" t="s">
+        <v>35</v>
+      </c>
+      <c r="C42">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
         <v>15</v>
       </c>
-      <c r="B26">
+      <c r="B43" t="s">
+        <v>64</v>
+      </c>
+      <c r="C43">
         <v>224</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>16</v>
-      </c>
-      <c r="B27">
-        <v>27480</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>17</v>
-      </c>
-      <c r="B28">
-        <v>17166</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>18</v>
-      </c>
-      <c r="B29">
-        <v>16771</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>19</v>
-      </c>
-      <c r="B30">
-        <v>6113</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>20</v>
-      </c>
-      <c r="B31">
-        <v>3323</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>21</v>
-      </c>
-      <c r="B32">
-        <v>1801</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>22</v>
-      </c>
-      <c r="B33">
-        <v>5034</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>23</v>
-      </c>
-      <c r="B34">
-        <v>788</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>24</v>
-      </c>
-      <c r="B35">
-        <v>11821</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>25</v>
-      </c>
-      <c r="B36">
-        <v>12573</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>26</v>
-      </c>
-      <c r="B37">
-        <v>1264</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>27</v>
-      </c>
-      <c r="B38">
-        <v>28471</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>28</v>
-      </c>
-      <c r="B39">
-        <v>18208</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>29</v>
-      </c>
-      <c r="B40">
-        <v>18208</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>30</v>
-      </c>
-      <c r="B41">
-        <v>5704</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>31</v>
-      </c>
-      <c r="B42">
-        <v>6317</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>32</v>
-      </c>
-      <c r="B43">
-        <v>10090</v>
-      </c>
-    </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C43">
+    <sortCondition descending="1" ref="C2:C43"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>